<commit_message>
output judge gpt guideline
</commit_message>
<xml_diff>
--- a/output/metrics/metrics_gpt_judge_bge_m3_guideline.xlsx
+++ b/output/metrics/metrics_gpt_judge_bge_m3_guideline.xlsx
@@ -485,31 +485,31 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4820924337854682</v>
+        <v>0.5371692965393693</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8106995884773662</v>
+        <v>0.898</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6877914951989026</v>
+        <v>0.7662666666666667</v>
       </c>
       <c r="I2" t="n">
-        <v>32.83950617283951</v>
+        <v>36.88</v>
       </c>
       <c r="J2" t="n">
-        <v>31.97530864197531</v>
+        <v>35</v>
       </c>
       <c r="K2" t="n">
-        <v>35.18518518518518</v>
+        <v>28.12</v>
       </c>
     </row>
     <row r="3">
@@ -524,31 +524,31 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2425</v>
+        <v>2500</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3493150745719905</v>
+        <v>0.3880411642607319</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5452674897119342</v>
+        <v>0.61</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4085048010973937</v>
+        <v>0.4548666666666667</v>
       </c>
       <c r="I3" t="n">
-        <v>18.63917525773196</v>
+        <v>20.96</v>
       </c>
       <c r="J3" t="n">
-        <v>41.03092783505154</v>
+        <v>44.76</v>
       </c>
       <c r="K3" t="n">
-        <v>40.32989690721649</v>
+        <v>34.28</v>
       </c>
     </row>
     <row r="4">
@@ -563,31 +563,31 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>2425</v>
+        <v>2500</v>
       </c>
       <c r="F4" t="n">
-        <v>0.355289419238527</v>
+        <v>0.3918585094941918</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5864197530864198</v>
+        <v>0.658</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4272976680384088</v>
+        <v>0.4704666666666666</v>
       </c>
       <c r="I4" t="n">
-        <v>19.50515463917526</v>
+        <v>21.76</v>
       </c>
       <c r="J4" t="n">
-        <v>40.28865979381443</v>
+        <v>43.84</v>
       </c>
       <c r="K4" t="n">
-        <v>40.20618556701031</v>
+        <v>34.4</v>
       </c>
     </row>
     <row r="5">
@@ -602,31 +602,31 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3742889928176292</v>
+        <v>0.4127129262202721</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5925925925925926</v>
+        <v>0.662</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4542524005486968</v>
+        <v>0.5060999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>21.11111111111111</v>
+        <v>23.56</v>
       </c>
       <c r="J5" t="n">
-        <v>39.62962962962963</v>
+        <v>42.76</v>
       </c>
       <c r="K5" t="n">
-        <v>39.25925925925926</v>
+        <v>33.68</v>
       </c>
     </row>
     <row r="6">
@@ -641,31 +641,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3668352817667968</v>
+        <v>0.4050578096376825</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.626</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4183470507544582</v>
+        <v>0.4649666666666667</v>
       </c>
       <c r="I6" t="n">
-        <v>20.24691358024691</v>
+        <v>22.64</v>
       </c>
       <c r="J6" t="n">
-        <v>42.05761316872428</v>
+        <v>45.72</v>
       </c>
       <c r="K6" t="n">
-        <v>37.69547325102881</v>
+        <v>31.64</v>
       </c>
     </row>
     <row r="7">
@@ -680,31 +680,31 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>2425</v>
+        <v>2500</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3656323770382033</v>
+        <v>0.4011271838470364</v>
       </c>
       <c r="G7" t="n">
-        <v>0.565843621399177</v>
+        <v>0.62</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4300754458161866</v>
+        <v>0.4708666666666667</v>
       </c>
       <c r="I7" t="n">
-        <v>20.41237113402062</v>
+        <v>22.56</v>
       </c>
       <c r="J7" t="n">
-        <v>40.74226804123711</v>
+        <v>44.24</v>
       </c>
       <c r="K7" t="n">
-        <v>38.84536082474227</v>
+        <v>33.2</v>
       </c>
     </row>
     <row r="8">
@@ -719,31 +719,31 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>2425</v>
+        <v>2500</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3810662796726517</v>
+        <v>0.4204224102730001</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5720164609053497</v>
+        <v>0.628</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4451646090534979</v>
+        <v>0.4896666666666666</v>
       </c>
       <c r="I8" t="n">
-        <v>22.18556701030928</v>
+        <v>24.44</v>
       </c>
       <c r="J8" t="n">
-        <v>39.62886597938144</v>
+        <v>43.72</v>
       </c>
       <c r="K8" t="n">
-        <v>38.18556701030928</v>
+        <v>31.84</v>
       </c>
     </row>
     <row r="9">
@@ -758,31 +758,31 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3689200070524993</v>
+        <v>0.4048051442160434</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5823045267489712</v>
+        <v>0.65</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4308299039780521</v>
+        <v>0.4727666666666667</v>
       </c>
       <c r="I9" t="n">
-        <v>20.61728395061728</v>
+        <v>22.88</v>
       </c>
       <c r="J9" t="n">
-        <v>41.81069958847737</v>
+        <v>45.4</v>
       </c>
       <c r="K9" t="n">
-        <v>37.57201646090535</v>
+        <v>31.72</v>
       </c>
     </row>
     <row r="10">
@@ -797,31 +797,31 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3542845948392848</v>
+        <v>0.3879173732894229</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5679012345679012</v>
+        <v>0.62</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4450274348422497</v>
+        <v>0.4811333333333333</v>
       </c>
       <c r="I10" t="n">
-        <v>19.58847736625514</v>
+        <v>21.44</v>
       </c>
       <c r="J10" t="n">
-        <v>38.35390946502058</v>
+        <v>42.48</v>
       </c>
       <c r="K10" t="n">
-        <v>42.05761316872428</v>
+        <v>36.08</v>
       </c>
     </row>
     <row r="11">
@@ -836,31 +836,31 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4207514886869352</v>
+        <v>0.4597675987414608</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6049382716049383</v>
+        <v>0.666</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4727366255144033</v>
+        <v>0.5168333333333334</v>
       </c>
       <c r="I11" t="n">
-        <v>27.03703703703704</v>
+        <v>29.8</v>
       </c>
       <c r="J11" t="n">
-        <v>37.48971193415638</v>
+        <v>40.68</v>
       </c>
       <c r="K11" t="n">
-        <v>35.47325102880659</v>
+        <v>29.52</v>
       </c>
     </row>
     <row r="12">
@@ -875,31 +875,31 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4148473736353847</v>
+        <v>0.4530627591226635</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5699588477366255</v>
+        <v>0.628</v>
       </c>
       <c r="H12" t="n">
-        <v>0.46059670781893</v>
+        <v>0.4961333333333333</v>
       </c>
       <c r="I12" t="n">
-        <v>25.67901234567901</v>
+        <v>28.24</v>
       </c>
       <c r="J12" t="n">
-        <v>40.16460905349794</v>
+        <v>43.91999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>34.15637860082305</v>
+        <v>27.84</v>
       </c>
     </row>
     <row r="13">
@@ -914,31 +914,31 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3615945688959601</v>
+        <v>0.4010859205461245</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5843621399176955</v>
+        <v>0.654</v>
       </c>
       <c r="H13" t="n">
-        <v>0.4470850480109739</v>
+        <v>0.4954333333333333</v>
       </c>
       <c r="I13" t="n">
-        <v>20.2880658436214</v>
+        <v>22.76</v>
       </c>
       <c r="J13" t="n">
-        <v>38.559670781893</v>
+        <v>42.44</v>
       </c>
       <c r="K13" t="n">
-        <v>41.1522633744856</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="14">
@@ -953,31 +953,31 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F14" t="n">
-        <v>0.3737383431167694</v>
+        <v>0.4091231347512005</v>
       </c>
       <c r="G14" t="n">
-        <v>0.5967078189300411</v>
+        <v>0.662</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4641975308641975</v>
+        <v>0.5089333333333333</v>
       </c>
       <c r="I14" t="n">
-        <v>20.69958847736626</v>
+        <v>22.84</v>
       </c>
       <c r="J14" t="n">
-        <v>40.24691358024691</v>
+        <v>43.8</v>
       </c>
       <c r="K14" t="n">
-        <v>39.05349794238683</v>
+        <v>33.36</v>
       </c>
     </row>
     <row r="15">
@@ -992,31 +992,31 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>2425</v>
+        <v>2500</v>
       </c>
       <c r="F15" t="n">
-        <v>0.352678334326635</v>
+        <v>0.3855881796491852</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5905349794238683</v>
+        <v>0.64</v>
       </c>
       <c r="H15" t="n">
-        <v>0.4205761316872428</v>
+        <v>0.4601333333333333</v>
       </c>
       <c r="I15" t="n">
-        <v>19.58762886597938</v>
+        <v>21.48</v>
       </c>
       <c r="J15" t="n">
-        <v>39.62886597938144</v>
+        <v>42.92</v>
       </c>
       <c r="K15" t="n">
-        <v>40.78350515463918</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="16">
@@ -1031,31 +1031,31 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F16" t="n">
-        <v>0.3570582185284665</v>
+        <v>0.3874439772580535</v>
       </c>
       <c r="G16" t="n">
-        <v>0.5823045267489712</v>
+        <v>0.636</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4303840877914952</v>
+        <v>0.4607</v>
       </c>
       <c r="I16" t="n">
-        <v>19.79423868312757</v>
+        <v>21.64</v>
       </c>
       <c r="J16" t="n">
-        <v>39.42386831275721</v>
+        <v>43.04</v>
       </c>
       <c r="K16" t="n">
-        <v>40.78189300411523</v>
+        <v>35.32</v>
       </c>
     </row>
     <row r="17">
@@ -1070,31 +1070,31 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>2426</v>
+        <v>2500</v>
       </c>
       <c r="F17" t="n">
-        <v>0.3060078831141748</v>
+        <v>0.3316265427856385</v>
       </c>
       <c r="G17" t="n">
-        <v>0.4567901234567901</v>
+        <v>0.502</v>
       </c>
       <c r="H17" t="n">
-        <v>0.3507201646090535</v>
+        <v>0.3835666666666667</v>
       </c>
       <c r="I17" t="n">
-        <v>15.62242374278648</v>
+        <v>17.04</v>
       </c>
       <c r="J17" t="n">
-        <v>38.12860676009893</v>
+        <v>41</v>
       </c>
       <c r="K17" t="n">
-        <v>46.24896949711459</v>
+        <v>41.95999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -1109,31 +1109,31 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>2425</v>
+        <v>2500</v>
       </c>
       <c r="F18" t="n">
-        <v>0.3570874666056061</v>
+        <v>0.388222796781664</v>
       </c>
       <c r="G18" t="n">
-        <v>0.5370370370370371</v>
+        <v>0.602</v>
       </c>
       <c r="H18" t="n">
-        <v>0.4152263374485597</v>
+        <v>0.4506</v>
       </c>
       <c r="I18" t="n">
-        <v>18.96907216494845</v>
+        <v>20.6</v>
       </c>
       <c r="J18" t="n">
-        <v>41.64948453608248</v>
+        <v>45.56</v>
       </c>
       <c r="K18" t="n">
-        <v>39.38144329896907</v>
+        <v>33.84</v>
       </c>
     </row>
     <row r="19">
@@ -1148,31 +1148,31 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F19" t="n">
-        <v>0.2946979839679472</v>
+        <v>0.3180377546171546</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4259259259259259</v>
+        <v>0.466</v>
       </c>
       <c r="H19" t="n">
-        <v>0.3141975308641975</v>
+        <v>0.3409666666666667</v>
       </c>
       <c r="I19" t="n">
-        <v>14.40329218106996</v>
+        <v>15.56</v>
       </c>
       <c r="J19" t="n">
-        <v>38.97119341563786</v>
+        <v>42.16</v>
       </c>
       <c r="K19" t="n">
-        <v>46.62551440329218</v>
+        <v>42.28</v>
       </c>
     </row>
     <row r="20">
@@ -1187,31 +1187,31 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F20" t="n">
-        <v>0.3741970212647096</v>
+        <v>0.4092017804715591</v>
       </c>
       <c r="G20" t="n">
-        <v>0.588477366255144</v>
+        <v>0.648</v>
       </c>
       <c r="H20" t="n">
-        <v>0.4471536351165981</v>
+        <v>0.4935</v>
       </c>
       <c r="I20" t="n">
-        <v>21.60493827160494</v>
+        <v>23.68</v>
       </c>
       <c r="J20" t="n">
-        <v>38.97119341563786</v>
+        <v>42.64</v>
       </c>
       <c r="K20" t="n">
-        <v>39.42386831275721</v>
+        <v>33.68</v>
       </c>
     </row>
     <row r="21">
@@ -1226,31 +1226,31 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>2430</v>
+        <v>2500</v>
       </c>
       <c r="F21" t="n">
-        <v>0.4950436549785256</v>
+        <v>0.5427184017839933</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5946502057613169</v>
+        <v>0.654</v>
       </c>
       <c r="H21" t="n">
-        <v>0.4795610425240055</v>
+        <v>0.5259666666666667</v>
       </c>
       <c r="I21" t="n">
-        <v>36.5843621399177</v>
+        <v>40.12</v>
       </c>
       <c r="J21" t="n">
-        <v>35.92592592592593</v>
+        <v>39.32</v>
       </c>
       <c r="K21" t="n">
-        <v>27.48971193415638</v>
+        <v>20.56</v>
       </c>
     </row>
     <row r="22">
@@ -1265,31 +1265,31 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>2425</v>
+        <v>2500</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3403258759556265</v>
+        <v>0.3677884909446581</v>
       </c>
       <c r="G22" t="n">
-        <v>0.5267489711934157</v>
+        <v>0.578</v>
       </c>
       <c r="H22" t="n">
-        <v>0.3926611796982167</v>
+        <v>0.4152999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>18.55670103092784</v>
+        <v>20.04</v>
       </c>
       <c r="J22" t="n">
-        <v>39.25773195876289</v>
+        <v>43.16</v>
       </c>
       <c r="K22" t="n">
-        <v>42.18556701030928</v>
+        <v>36.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>